<commit_message>
update: run full-scale whitelisted Henderson PDF override and packing
</commit_message>
<xml_diff>
--- a/files/九龙-佐敦-高临.xlsx
+++ b/files/九龙-佐敦-高临.xlsx
@@ -122,7 +122,8 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
-      <color rgb="00002060"/>
+      <b val="1"/>
+      <color rgb="00004D00"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -267,7 +268,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8633,7 +8634,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>已定价未售</t>
+          <t>在售</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
@@ -18155,12 +18156,12 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
@@ -18242,7 +18243,7 @@
           <t>A | 1452呎 (4+房)
 招标单位
 -
-(已定价未售)</t>
+(在售)</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr"/>

</xml_diff>